<commit_message>
BWI sync — 2026-06-06 13:48 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Angola.xlsx
+++ b/BWI/bestwine_output/bestwine_Angola.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA22"/>
+  <dimension ref="A1:AA24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2533,6 +2533,208 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Angola</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>nº 61 Município de Ingombota</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>https://multiafrica.com</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>geral@multiafrica.com</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr"/>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/grupo-multi%C3%A1frica/</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/people/Multiáfrica/100088549989829</t>
+        </is>
+      </c>
+      <c r="T23" s="2" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/multiafrica</t>
+        </is>
+      </c>
+      <c r="U23" s="2" t="inlineStr"/>
+      <c r="V23" s="2" t="inlineStr"/>
+      <c r="W23" s="2" t="inlineStr">
+        <is>
+          <t>Diogo Miranda Alves</t>
+        </is>
+      </c>
+      <c r="X23" s="2" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+      <c r="Y23" s="2" t="inlineStr"/>
+      <c r="Z23" s="2" t="inlineStr"/>
+      <c r="AA23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/diogo-miranda-alves-05185a90/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Angola</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>nº 61 Município de Ingombota</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>https://multiafrica.com</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>geral@multiafrica.com</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr"/>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr"/>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/grupo-multi%C3%A1frica/</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/people/Multiáfrica/100088549989829</t>
+        </is>
+      </c>
+      <c r="T24" s="2" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/multiafrica</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr"/>
+      <c r="V24" s="2" t="inlineStr"/>
+      <c r="W24" s="2" t="inlineStr">
+        <is>
+          <t>Roberto Lopes</t>
+        </is>
+      </c>
+      <c r="X24" s="2" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
+      <c r="Y24" s="2" t="inlineStr"/>
+      <c r="Z24" s="2" t="inlineStr"/>
+      <c r="AA24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/roberto-lopes-4a458793/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BWI sync — 2026-06-08 13:11 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Angola.xlsx
+++ b/BWI/bestwine_output/bestwine_Angola.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA24"/>
+  <dimension ref="A1:AA26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2735,6 +2735,208 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Angola</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>nº 61 Município de Ingombota</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>https://multiafrica.com</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>geral@multiafrica.com</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr"/>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/grupo-multi%C3%A1frica/</t>
+        </is>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/people/Multiáfrica/100088549989829</t>
+        </is>
+      </c>
+      <c r="T25" s="2" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/multiafrica</t>
+        </is>
+      </c>
+      <c r="U25" s="2" t="inlineStr"/>
+      <c r="V25" s="2" t="inlineStr"/>
+      <c r="W25" s="2" t="inlineStr">
+        <is>
+          <t>Diogo Miranda Alves</t>
+        </is>
+      </c>
+      <c r="X25" s="2" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+      <c r="Y25" s="2" t="inlineStr"/>
+      <c r="Z25" s="2" t="inlineStr"/>
+      <c r="AA25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/diogo-miranda-alves-05185a90/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Angola</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>nº 61 Município de Ingombota</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>https://multiafrica.com</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>geral@multiafrica.com</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/grupo-multi%C3%A1frica/</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/people/Multiáfrica/100088549989829</t>
+        </is>
+      </c>
+      <c r="T26" s="2" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/multiafrica</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr"/>
+      <c r="V26" s="2" t="inlineStr"/>
+      <c r="W26" s="2" t="inlineStr">
+        <is>
+          <t>Roberto Lopes</t>
+        </is>
+      </c>
+      <c r="X26" s="2" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
+      <c r="Y26" s="2" t="inlineStr"/>
+      <c r="Z26" s="2" t="inlineStr"/>
+      <c r="AA26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/roberto-lopes-4a458793/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BWI sync — 2026-06-15 15:30 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Angola.xlsx
+++ b/BWI/bestwine_output/bestwine_Angola.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA26"/>
+  <dimension ref="A1:AA28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2937,6 +2937,208 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Angola</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>nº 61 Município de Ingombota</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>https://multiafrica.com</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>geral@multiafrica.com</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/grupo-multi%C3%A1frica/</t>
+        </is>
+      </c>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/people/Multiáfrica/100088549989829</t>
+        </is>
+      </c>
+      <c r="T27" s="2" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/multiafrica</t>
+        </is>
+      </c>
+      <c r="U27" s="2" t="inlineStr"/>
+      <c r="V27" s="2" t="inlineStr"/>
+      <c r="W27" s="2" t="inlineStr">
+        <is>
+          <t>Diogo Miranda Alves</t>
+        </is>
+      </c>
+      <c r="X27" s="2" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+      <c r="Y27" s="2" t="inlineStr"/>
+      <c r="Z27" s="2" t="inlineStr"/>
+      <c r="AA27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/diogo-miranda-alves-05185a90/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Angola</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>nº 61 Município de Ingombota</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>https://multiafrica.com</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>geral@multiafrica.com</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/grupo-multi%C3%A1frica/</t>
+        </is>
+      </c>
+      <c r="S28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/people/Multiáfrica/100088549989829</t>
+        </is>
+      </c>
+      <c r="T28" s="2" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/multiafrica</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr"/>
+      <c r="V28" s="2" t="inlineStr"/>
+      <c r="W28" s="2" t="inlineStr">
+        <is>
+          <t>Roberto Lopes</t>
+        </is>
+      </c>
+      <c r="X28" s="2" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
+      <c r="Y28" s="2" t="inlineStr"/>
+      <c r="Z28" s="2" t="inlineStr"/>
+      <c r="AA28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/roberto-lopes-4a458793/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BWI sync — 2026-06-22 15:05 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Angola.xlsx
+++ b/BWI/bestwine_output/bestwine_Angola.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA28"/>
+  <dimension ref="A1:AA30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3139,6 +3139,208 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Angola</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>nº 61 Município de Ingombota</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>https://multiafrica.com</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>geral@multiafrica.com</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr"/>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="inlineStr"/>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/grupo-multi%C3%A1frica/</t>
+        </is>
+      </c>
+      <c r="S29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/people/Multiáfrica/100088549989829</t>
+        </is>
+      </c>
+      <c r="T29" s="2" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/multiafrica</t>
+        </is>
+      </c>
+      <c r="U29" s="2" t="inlineStr"/>
+      <c r="V29" s="2" t="inlineStr"/>
+      <c r="W29" s="2" t="inlineStr">
+        <is>
+          <t>Diogo Miranda Alves</t>
+        </is>
+      </c>
+      <c r="X29" s="2" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+      <c r="Y29" s="2" t="inlineStr"/>
+      <c r="Z29" s="2" t="inlineStr"/>
+      <c r="AA29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/diogo-miranda-alves-05185a90/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Multiafrica - Comercio Restauracao E Hotelaria, Lda</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Angola</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Luanda</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>nº 61 Município de Ingombota</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>https://multiafrica.com</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>geral@multiafrica.com</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr"/>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr"/>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/grupo-multi%C3%A1frica/</t>
+        </is>
+      </c>
+      <c r="S30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/people/Multiáfrica/100088549989829</t>
+        </is>
+      </c>
+      <c r="T30" s="2" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/multiafrica</t>
+        </is>
+      </c>
+      <c r="U30" s="2" t="inlineStr"/>
+      <c r="V30" s="2" t="inlineStr"/>
+      <c r="W30" s="2" t="inlineStr">
+        <is>
+          <t>Roberto Lopes</t>
+        </is>
+      </c>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
+      <c r="Y30" s="2" t="inlineStr"/>
+      <c r="Z30" s="2" t="inlineStr"/>
+      <c r="AA30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/roberto-lopes-4a458793/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>